<commit_message>
Verifica settimanale (parziale): deduplica cross-file, 16 duplicati marcati
Marcati come duplicati (nota [DUPLICATO]) i record di distributori già
presenti in un file precedente, individuati per corrispondenza esatta di
dominio sito web o ragione sociale normalizzata. Le righe canoniche (file
più vecchio) restano invariate. Run ancora in corso: doppio controllo
WebSearch sui record non duplicati in elaborazione.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158TzxJdksXSnffhmC7YjQN
</commit_message>
<xml_diff>
--- a/output/2026-08-31_09_Italia_Toscana_Depolverazione_Trattamento_aria.xlsx
+++ b/output/2026-08-31_09_Italia_Toscana_Depolverazione_Trattamento_aria.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Impianti di aspirazione industriale, filtrazione aria, depolverazione; attiva dal 1979.</t>
+          <t>Impianti di aspirazione industriale, filtrazione aria, depolverazione; attiva dal 1979. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Impianti di aspirazione industriale e canalizzazioni.</t>
+          <t>Impianti di aspirazione industriale e canalizzazioni. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Azienda dal 1990 (esperienza dal 1970), impianti di aspirazione/depolverazione/filtrazione fumi e polveri. NOTA: le voci grezze 'Toscana Impianti Srl' (Pisa) e 'Toscana Impianti Srl' (Grosseto) risultano riferirsi allo stesso sito/contatti di questa azienda: deduplicate qui.</t>
+          <t>Azienda dal 1990 (esperienza dal 1970), impianti di aspirazione/depolverazione/filtrazione fumi e polveri. NOTA: le voci grezze 'Toscana Impianti Srl' (Pisa) e 'Toscana Impianti Srl' (Grosseto) risultano riferirsi allo stesso sito/contatti di questa azienda: deduplicate qui. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Aspirazione industriale, trattamento fumi di saldatura, filtri a maniche/cartucce/carboni attivi.</t>
+          <t>Aspirazione industriale, trattamento fumi di saldatura, filtri a maniche/cartucce/carboni attivi. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Vendita/noleggio aspiratori industriali (liquidi/polveri); attiva dal 1980.</t>
+          <t>Vendita/noleggio aspiratori industriali (liquidi/polveri); attiva dal 1980. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Distributore aspiratori industriali Coynco. IMPORTANTE: fonti web indicano che distribuisce anche prodotti a marchio DU-PUY - possibile rivenditore gia' attivo del brand, verificare con priorita'.</t>
+          <t>Distributore aspiratori industriali Coynco. IMPORTANTE: fonti web indicano che distribuisce anche prodotti a marchio DU-PUY - possibile rivenditore gia' attivo del brand, verificare con priorita'. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">

</xml_diff>